<commit_message>
test(#353): vaciar los costos del caso 07 del dataset dorado
El original es un formulario ya costeado: sus costos y tarifas se vacían en la réplica,
como llega una licitación (igual que las tarifas del caso 05).
</commit_message>
<xml_diff>
--- a/tests/evaluacion-ia/dataset/casos/caso_07_cliente_d_impo_expo.xlsx
+++ b/tests/evaluacion-ia/dataset/casos/caso_07_cliente_d_impo_expo.xlsx
@@ -785,9 +785,7 @@
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="8" t="n"/>
-      <c r="H11" s="9" t="n">
-        <v>2705000</v>
-      </c>
+      <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="9" t="n"/>
@@ -817,9 +815,7 @@
       </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="8" t="n"/>
-      <c r="H12" s="9" t="n">
-        <v>2284000</v>
-      </c>
+      <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="9" t="n"/>
@@ -849,9 +845,7 @@
       </c>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="8" t="n"/>
-      <c r="H13" s="9" t="n">
-        <v>2286000</v>
-      </c>
+      <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="n"/>
@@ -881,9 +875,7 @@
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="8" t="n"/>
-      <c r="H14" s="9" t="n">
-        <v>6477000</v>
-      </c>
+      <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
       <c r="J14" s="9" t="n"/>
       <c r="K14" s="9" t="n"/>
@@ -913,9 +905,7 @@
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="8" t="n"/>
-      <c r="H15" s="9" t="n">
-        <v>4069000</v>
-      </c>
+      <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
@@ -945,9 +935,7 @@
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="8" t="n"/>
-      <c r="H16" s="9" t="n">
-        <v>4565000</v>
-      </c>
+      <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
       <c r="J16" s="9" t="n"/>
       <c r="K16" s="9" t="n"/>
@@ -977,9 +965,7 @@
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="8" t="n"/>
-      <c r="H17" s="9" t="n">
-        <v>3633000</v>
-      </c>
+      <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="9" t="n"/>
@@ -1009,9 +995,7 @@
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="8" t="n"/>
-      <c r="H18" s="9" t="n">
-        <v>3590000</v>
-      </c>
+      <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="9" t="n"/>
@@ -1041,9 +1025,7 @@
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="8" t="n"/>
-      <c r="H19" s="9" t="n">
-        <v>4988000</v>
-      </c>
+      <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="9" t="n"/>
@@ -1073,9 +1055,7 @@
       </c>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="8" t="n"/>
-      <c r="H20" s="9" t="n">
-        <v>3853000</v>
-      </c>
+      <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
       <c r="J20" s="9" t="n"/>
       <c r="K20" s="9" t="n"/>
@@ -1105,9 +1085,7 @@
       </c>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="8" t="n"/>
-      <c r="H21" s="9" t="n">
-        <v>6624000</v>
-      </c>
+      <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
       <c r="J21" s="9" t="n"/>
       <c r="K21" s="9" t="n"/>
@@ -1123,7 +1101,7 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -1137,9 +1115,7 @@
       </c>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="8" t="n"/>
-      <c r="H22" s="9" t="n">
-        <v>3532000</v>
-      </c>
+      <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="9" t="n"/>
@@ -1155,7 +1131,7 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
@@ -1169,9 +1145,7 @@
       </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="8" t="n"/>
-      <c r="H23" s="9" t="n">
-        <v>5097000</v>
-      </c>
+      <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="9" t="n"/>
       <c r="K23" s="9" t="n"/>
@@ -1187,7 +1161,7 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
@@ -1201,9 +1175,7 @@
       </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="8" t="n"/>
-      <c r="H24" s="9" t="n">
-        <v>5486000</v>
-      </c>
+      <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="9" t="n"/>
@@ -1219,7 +1191,7 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
@@ -1233,9 +1205,7 @@
       </c>
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="8" t="n"/>
-      <c r="H25" s="9" t="n">
-        <v>3658000</v>
-      </c>
+      <c r="H25" s="9" t="n"/>
       <c r="I25" s="9" t="n"/>
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="9" t="n"/>
@@ -1251,7 +1221,7 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
@@ -1265,9 +1235,7 @@
       </c>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="8" t="n"/>
-      <c r="H26" s="9" t="n">
-        <v>3840000</v>
-      </c>
+      <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="9" t="n"/>
       <c r="K26" s="9" t="n"/>
@@ -1283,7 +1251,7 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
@@ -1297,9 +1265,7 @@
       </c>
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="8" t="n"/>
-      <c r="H27" s="9" t="n">
-        <v>6446000</v>
-      </c>
+      <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="9" t="n"/>
@@ -1315,7 +1281,7 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
@@ -1329,9 +1295,7 @@
       </c>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="8" t="n"/>
-      <c r="H28" s="9" t="n">
-        <v>3991000</v>
-      </c>
+      <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="9" t="n"/>
       <c r="K28" s="9" t="n"/>
@@ -1347,7 +1311,7 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -1361,9 +1325,7 @@
       </c>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="8" t="n"/>
-      <c r="H29" s="9" t="n">
-        <v>3588000</v>
-      </c>
+      <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="J29" s="9" t="n"/>
       <c r="K29" s="9" t="n"/>
@@ -1379,7 +1341,7 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
@@ -1393,9 +1355,7 @@
       </c>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="8" t="n"/>
-      <c r="H30" s="9" t="n">
-        <v>5790000</v>
-      </c>
+      <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="9" t="n"/>
       <c r="K30" s="9" t="n"/>
@@ -1411,7 +1371,7 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -1425,9 +1385,7 @@
       </c>
       <c r="F31" s="5" t="n"/>
       <c r="G31" s="8" t="n"/>
-      <c r="H31" s="9" t="n">
-        <v>4723000</v>
-      </c>
+      <c r="H31" s="9" t="n"/>
       <c r="I31" s="9" t="n"/>
       <c r="J31" s="9" t="n"/>
       <c r="K31" s="9" t="n"/>
@@ -1443,7 +1401,7 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>Chimichagua-Morroa</t>
+          <t>San Lorenzo-Morroa</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -1457,9 +1415,7 @@
       </c>
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="8" t="n"/>
-      <c r="H32" s="9" t="n">
-        <v>7919000</v>
-      </c>
+      <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
       <c r="J32" s="9" t="n"/>
       <c r="K32" s="9" t="n"/>
@@ -1489,9 +1445,7 @@
       </c>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="8" t="n"/>
-      <c r="H33" s="9" t="n">
-        <v>2636000</v>
-      </c>
+      <c r="H33" s="9" t="n"/>
       <c r="I33" s="9" t="n"/>
       <c r="J33" s="9" t="n"/>
       <c r="K33" s="9" t="n"/>
@@ -1521,9 +1475,7 @@
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="8" t="n"/>
-      <c r="H34" s="9" t="n">
-        <v>2689000</v>
-      </c>
+      <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="9" t="n"/>
       <c r="K34" s="9" t="n"/>
@@ -1553,9 +1505,7 @@
       </c>
       <c r="F35" s="5" t="n"/>
       <c r="G35" s="8" t="n"/>
-      <c r="H35" s="9" t="n">
-        <v>4358000</v>
-      </c>
+      <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="9" t="n"/>
       <c r="K35" s="9" t="n"/>
@@ -1585,9 +1535,7 @@
       </c>
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="8" t="n"/>
-      <c r="H36" s="9" t="n">
-        <v>3737000</v>
-      </c>
+      <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="9" t="n"/>
       <c r="K36" s="9" t="n"/>
@@ -1617,9 +1565,7 @@
       </c>
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="8" t="n"/>
-      <c r="H37" s="9" t="n">
-        <v>6396000</v>
-      </c>
+      <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="J37" s="9" t="n"/>
       <c r="K37" s="9" t="n"/>
@@ -1649,9 +1595,7 @@
       </c>
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="8" t="n"/>
-      <c r="H38" s="9" t="n">
-        <v>4748000</v>
-      </c>
+      <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
       <c r="J38" s="9" t="n"/>
       <c r="K38" s="9" t="n"/>
@@ -1681,9 +1625,7 @@
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="8" t="n"/>
-      <c r="H39" s="9" t="n">
-        <v>2344000</v>
-      </c>
+      <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="9" t="n"/>
       <c r="K39" s="9" t="n"/>
@@ -1713,9 +1655,7 @@
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="8" t="n"/>
-      <c r="H40" s="9" t="n">
-        <v>3583000</v>
-      </c>
+      <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
       <c r="J40" s="9" t="n"/>
       <c r="K40" s="9" t="n"/>
@@ -1745,9 +1685,7 @@
       </c>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="8" t="n"/>
-      <c r="H41" s="9" t="n">
-        <v>6627000</v>
-      </c>
+      <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="9" t="n"/>
       <c r="K41" s="9" t="n"/>
@@ -1777,9 +1715,7 @@
       </c>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="8" t="n"/>
-      <c r="H42" s="9" t="n">
-        <v>6526000</v>
-      </c>
+      <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
       <c r="J42" s="9" t="n"/>
       <c r="K42" s="9" t="n"/>
@@ -1809,9 +1745,7 @@
       </c>
       <c r="F43" s="5" t="n"/>
       <c r="G43" s="8" t="n"/>
-      <c r="H43" s="9" t="n">
-        <v>3702000</v>
-      </c>
+      <c r="H43" s="9" t="n"/>
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="9" t="n"/>
       <c r="K43" s="9" t="n"/>
@@ -1827,7 +1761,7 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
@@ -1841,9 +1775,7 @@
       </c>
       <c r="F44" s="5" t="n"/>
       <c r="G44" s="8" t="n"/>
-      <c r="H44" s="9" t="n">
-        <v>4057000</v>
-      </c>
+      <c r="H44" s="9" t="n"/>
       <c r="I44" s="9" t="n"/>
       <c r="J44" s="9" t="n"/>
       <c r="K44" s="9" t="n"/>
@@ -1859,7 +1791,7 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -1873,9 +1805,7 @@
       </c>
       <c r="F45" s="5" t="n"/>
       <c r="G45" s="8" t="n"/>
-      <c r="H45" s="9" t="n">
-        <v>5521000</v>
-      </c>
+      <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n"/>
       <c r="J45" s="9" t="n"/>
       <c r="K45" s="9" t="n"/>
@@ -1891,7 +1821,7 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
@@ -1905,9 +1835,7 @@
       </c>
       <c r="F46" s="5" t="n"/>
       <c r="G46" s="8" t="n"/>
-      <c r="H46" s="9" t="n">
-        <v>4152000</v>
-      </c>
+      <c r="H46" s="9" t="n"/>
       <c r="I46" s="9" t="n"/>
       <c r="J46" s="9" t="n"/>
       <c r="K46" s="9" t="n"/>
@@ -1923,7 +1851,7 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
@@ -1937,9 +1865,7 @@
       </c>
       <c r="F47" s="5" t="n"/>
       <c r="G47" s="8" t="n"/>
-      <c r="H47" s="9" t="n">
-        <v>4505000</v>
-      </c>
+      <c r="H47" s="9" t="n"/>
       <c r="I47" s="9" t="n"/>
       <c r="J47" s="9" t="n"/>
       <c r="K47" s="9" t="n"/>
@@ -1955,7 +1881,7 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C48" s="5" t="n">
@@ -1969,9 +1895,7 @@
       </c>
       <c r="F48" s="5" t="n"/>
       <c r="G48" s="8" t="n"/>
-      <c r="H48" s="9" t="n">
-        <v>5998000</v>
-      </c>
+      <c r="H48" s="9" t="n"/>
       <c r="I48" s="9" t="n"/>
       <c r="J48" s="9" t="n"/>
       <c r="K48" s="9" t="n"/>
@@ -1987,7 +1911,7 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C49" s="5" t="n">
@@ -2001,9 +1925,7 @@
       </c>
       <c r="F49" s="5" t="n"/>
       <c r="G49" s="8" t="n"/>
-      <c r="H49" s="9" t="n">
-        <v>7629000</v>
-      </c>
+      <c r="H49" s="9" t="n"/>
       <c r="I49" s="9" t="n"/>
       <c r="J49" s="9" t="n"/>
       <c r="K49" s="9" t="n"/>
@@ -2019,7 +1941,7 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
@@ -2033,9 +1955,7 @@
       </c>
       <c r="F50" s="5" t="n"/>
       <c r="G50" s="8" t="n"/>
-      <c r="H50" s="9" t="n">
-        <v>4591000</v>
-      </c>
+      <c r="H50" s="9" t="n"/>
       <c r="I50" s="9" t="n"/>
       <c r="J50" s="9" t="n"/>
       <c r="K50" s="9" t="n"/>
@@ -2051,7 +1971,7 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
@@ -2065,9 +1985,7 @@
       </c>
       <c r="F51" s="5" t="n"/>
       <c r="G51" s="8" t="n"/>
-      <c r="H51" s="9" t="n">
-        <v>4400000</v>
-      </c>
+      <c r="H51" s="9" t="n"/>
       <c r="I51" s="9" t="n"/>
       <c r="J51" s="9" t="n"/>
       <c r="K51" s="9" t="n"/>
@@ -2083,7 +2001,7 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C52" s="5" t="n">
@@ -2097,9 +2015,7 @@
       </c>
       <c r="F52" s="5" t="n"/>
       <c r="G52" s="8" t="n"/>
-      <c r="H52" s="9" t="n">
-        <v>5192000</v>
-      </c>
+      <c r="H52" s="9" t="n"/>
       <c r="I52" s="9" t="n"/>
       <c r="J52" s="9" t="n"/>
       <c r="K52" s="9" t="n"/>
@@ -2115,7 +2031,7 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C53" s="5" t="n">
@@ -2129,9 +2045,7 @@
       </c>
       <c r="F53" s="5" t="n"/>
       <c r="G53" s="8" t="n"/>
-      <c r="H53" s="9" t="n">
-        <v>3834000</v>
-      </c>
+      <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
       <c r="J53" s="9" t="n"/>
       <c r="K53" s="9" t="n"/>
@@ -2147,7 +2061,7 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Chimichagua</t>
+          <t>Morroa-San Lorenzo</t>
         </is>
       </c>
       <c r="C54" s="5" t="n">
@@ -2161,9 +2075,7 @@
       </c>
       <c r="F54" s="5" t="n"/>
       <c r="G54" s="8" t="n"/>
-      <c r="H54" s="9" t="n">
-        <v>6449000</v>
-      </c>
+      <c r="H54" s="9" t="n"/>
       <c r="I54" s="9" t="n"/>
       <c r="J54" s="9" t="n"/>
       <c r="K54" s="9" t="n"/>
@@ -2179,7 +2091,7 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C55" s="5" t="n">
@@ -2193,9 +2105,7 @@
       </c>
       <c r="F55" s="5" t="n"/>
       <c r="G55" s="8" t="n"/>
-      <c r="H55" s="9" t="n">
-        <v>5841000</v>
-      </c>
+      <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
       <c r="J55" s="9" t="n"/>
       <c r="K55" s="9" t="n"/>
@@ -2211,7 +2121,7 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C56" s="5" t="n">
@@ -2225,9 +2135,7 @@
       </c>
       <c r="F56" s="5" t="n"/>
       <c r="G56" s="8" t="n"/>
-      <c r="H56" s="9" t="n">
-        <v>7721000</v>
-      </c>
+      <c r="H56" s="9" t="n"/>
       <c r="I56" s="9" t="n"/>
       <c r="J56" s="9" t="n"/>
       <c r="K56" s="9" t="n"/>
@@ -2243,7 +2151,7 @@
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C57" s="5" t="n">
@@ -2257,9 +2165,7 @@
       </c>
       <c r="F57" s="5" t="n"/>
       <c r="G57" s="8" t="n"/>
-      <c r="H57" s="9" t="n">
-        <v>3773000</v>
-      </c>
+      <c r="H57" s="9" t="n"/>
       <c r="I57" s="9" t="n"/>
       <c r="J57" s="9" t="n"/>
       <c r="K57" s="9" t="n"/>
@@ -2275,7 +2181,7 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C58" s="5" t="n">
@@ -2289,9 +2195,7 @@
       </c>
       <c r="F58" s="5" t="n"/>
       <c r="G58" s="8" t="n"/>
-      <c r="H58" s="9" t="n">
-        <v>7198000</v>
-      </c>
+      <c r="H58" s="9" t="n"/>
       <c r="I58" s="9" t="n"/>
       <c r="J58" s="9" t="n"/>
       <c r="K58" s="9" t="n"/>
@@ -2307,7 +2211,7 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C59" s="5" t="n">
@@ -2321,9 +2225,7 @@
       </c>
       <c r="F59" s="5" t="n"/>
       <c r="G59" s="8" t="n"/>
-      <c r="H59" s="9" t="n">
-        <v>10531000</v>
-      </c>
+      <c r="H59" s="9" t="n"/>
       <c r="I59" s="9" t="n"/>
       <c r="J59" s="9" t="n"/>
       <c r="K59" s="9" t="n"/>
@@ -2339,7 +2241,7 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C60" s="5" t="n">
@@ -2353,9 +2255,7 @@
       </c>
       <c r="F60" s="5" t="n"/>
       <c r="G60" s="8" t="n"/>
-      <c r="H60" s="9" t="n">
-        <v>7603000</v>
-      </c>
+      <c r="H60" s="9" t="n"/>
       <c r="I60" s="9" t="n"/>
       <c r="J60" s="9" t="n"/>
       <c r="K60" s="9" t="n"/>
@@ -2371,7 +2271,7 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C61" s="5" t="n">
@@ -2385,9 +2285,7 @@
       </c>
       <c r="F61" s="5" t="n"/>
       <c r="G61" s="8" t="n"/>
-      <c r="H61" s="9" t="n">
-        <v>4634000</v>
-      </c>
+      <c r="H61" s="9" t="n"/>
       <c r="I61" s="9" t="n"/>
       <c r="J61" s="9" t="n"/>
       <c r="K61" s="9" t="n"/>
@@ -2403,7 +2301,7 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C62" s="5" t="n">
@@ -2417,9 +2315,7 @@
       </c>
       <c r="F62" s="5" t="n"/>
       <c r="G62" s="8" t="n"/>
-      <c r="H62" s="9" t="n">
-        <v>7402000</v>
-      </c>
+      <c r="H62" s="9" t="n"/>
       <c r="I62" s="9" t="n"/>
       <c r="J62" s="9" t="n"/>
       <c r="K62" s="9" t="n"/>
@@ -2435,7 +2331,7 @@
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -2449,9 +2345,7 @@
       </c>
       <c r="F63" s="5" t="n"/>
       <c r="G63" s="8" t="n"/>
-      <c r="H63" s="9" t="n">
-        <v>5400000</v>
-      </c>
+      <c r="H63" s="9" t="n"/>
       <c r="I63" s="9" t="n"/>
       <c r="J63" s="9" t="n"/>
       <c r="K63" s="9" t="n"/>
@@ -2467,7 +2361,7 @@
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -2481,9 +2375,7 @@
       </c>
       <c r="F64" s="5" t="n"/>
       <c r="G64" s="8" t="n"/>
-      <c r="H64" s="9" t="n">
-        <v>8064000</v>
-      </c>
+      <c r="H64" s="9" t="n"/>
       <c r="I64" s="9" t="n"/>
       <c r="J64" s="9" t="n"/>
       <c r="K64" s="9" t="n"/>
@@ -2499,7 +2391,7 @@
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Cantagallo</t>
+          <t>Morroa-Lebrija</t>
         </is>
       </c>
       <c r="C65" s="5" t="n">
@@ -2513,9 +2405,7 @@
       </c>
       <c r="F65" s="5" t="n"/>
       <c r="G65" s="8" t="n"/>
-      <c r="H65" s="9" t="n">
-        <v>10802000</v>
-      </c>
+      <c r="H65" s="9" t="n"/>
       <c r="I65" s="9" t="n"/>
       <c r="J65" s="9" t="n"/>
       <c r="K65" s="9" t="n"/>
@@ -2531,7 +2421,7 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C66" s="5" t="n">
@@ -2561,7 +2451,7 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C67" s="5" t="n">
@@ -2591,7 +2481,7 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C68" s="5" t="n">
@@ -2621,7 +2511,7 @@
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C69" s="5" t="n">
@@ -2651,7 +2541,7 @@
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C70" s="5" t="n">
@@ -2681,7 +2571,7 @@
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C71" s="5" t="n">
@@ -2711,7 +2601,7 @@
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C72" s="5" t="n">
@@ -2741,7 +2631,7 @@
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C73" s="5" t="n">
@@ -2771,7 +2661,7 @@
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C74" s="5" t="n">
@@ -2801,7 +2691,7 @@
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C75" s="5" t="n">
@@ -2831,7 +2721,7 @@
       </c>
       <c r="B76" s="16" t="inlineStr">
         <is>
-          <t>Morroa-Rovira</t>
+          <t>Morroa-Chivolo</t>
         </is>
       </c>
       <c r="C76" s="5" t="n">

</xml_diff>